<commit_message>
Update aircraft cycles (2026-05-08T21:10:15.420Z)
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F21"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -619,9 +619,209 @@
         <v>0</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>2026-05-08</v>
+      </c>
+      <c r="B12">
+        <v>2026</v>
+      </c>
+      <c r="C12">
+        <v>19</v>
+      </c>
+      <c r="D12" t="str">
+        <v>CN-NMH</v>
+      </c>
+      <c r="E12" t="str">
+        <v>A320</v>
+      </c>
+      <c r="F12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>2026-05-08</v>
+      </c>
+      <c r="B13">
+        <v>2026</v>
+      </c>
+      <c r="C13">
+        <v>19</v>
+      </c>
+      <c r="D13" t="str">
+        <v>CN-NMI</v>
+      </c>
+      <c r="E13" t="str">
+        <v>A320</v>
+      </c>
+      <c r="F13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>2026-05-08</v>
+      </c>
+      <c r="B14">
+        <v>2026</v>
+      </c>
+      <c r="C14">
+        <v>19</v>
+      </c>
+      <c r="D14" t="str">
+        <v>CN-NMJ</v>
+      </c>
+      <c r="E14" t="str">
+        <v>A320</v>
+      </c>
+      <c r="F14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>2026-05-08</v>
+      </c>
+      <c r="B15">
+        <v>2026</v>
+      </c>
+      <c r="C15">
+        <v>19</v>
+      </c>
+      <c r="D15" t="str">
+        <v>CN-NML</v>
+      </c>
+      <c r="E15" t="str">
+        <v>A320</v>
+      </c>
+      <c r="F15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>2026-05-08</v>
+      </c>
+      <c r="B16">
+        <v>2026</v>
+      </c>
+      <c r="C16">
+        <v>19</v>
+      </c>
+      <c r="D16" t="str">
+        <v>CN-NMN</v>
+      </c>
+      <c r="E16" t="str">
+        <v>A320</v>
+      </c>
+      <c r="F16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>2026-05-08</v>
+      </c>
+      <c r="B17">
+        <v>2026</v>
+      </c>
+      <c r="C17">
+        <v>19</v>
+      </c>
+      <c r="D17" t="str">
+        <v>CN-NMO</v>
+      </c>
+      <c r="E17" t="str">
+        <v>A320</v>
+      </c>
+      <c r="F17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>2026-05-08</v>
+      </c>
+      <c r="B18">
+        <v>2026</v>
+      </c>
+      <c r="C18">
+        <v>19</v>
+      </c>
+      <c r="D18" t="str">
+        <v>CN-NMP</v>
+      </c>
+      <c r="E18" t="str">
+        <v>A320</v>
+      </c>
+      <c r="F18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>2026-05-08</v>
+      </c>
+      <c r="B19">
+        <v>2026</v>
+      </c>
+      <c r="C19">
+        <v>19</v>
+      </c>
+      <c r="D19" t="str">
+        <v>CN-NMQ</v>
+      </c>
+      <c r="E19" t="str">
+        <v>A320</v>
+      </c>
+      <c r="F19">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>2026-05-08</v>
+      </c>
+      <c r="B20">
+        <v>2026</v>
+      </c>
+      <c r="C20">
+        <v>19</v>
+      </c>
+      <c r="D20" t="str">
+        <v>CN-NMS</v>
+      </c>
+      <c r="E20" t="str">
+        <v>A320</v>
+      </c>
+      <c r="F20">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>2026-05-08</v>
+      </c>
+      <c r="B21">
+        <v>2026</v>
+      </c>
+      <c r="C21">
+        <v>19</v>
+      </c>
+      <c r="D21" t="str">
+        <v>CN-NMT</v>
+      </c>
+      <c r="E21" t="str">
+        <v>A320</v>
+      </c>
+      <c r="F21">
+        <v>9</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F21"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update aircraft cycles (2026-05-08T21:14:27.312Z)
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F31"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -819,9 +819,209 @@
         <v>9</v>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>2026-05-08</v>
+      </c>
+      <c r="B22">
+        <v>2026</v>
+      </c>
+      <c r="C22">
+        <v>19</v>
+      </c>
+      <c r="D22" t="str">
+        <v>CN-NMH</v>
+      </c>
+      <c r="E22" t="str">
+        <v>A320</v>
+      </c>
+      <c r="F22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>2026-05-08</v>
+      </c>
+      <c r="B23">
+        <v>2026</v>
+      </c>
+      <c r="C23">
+        <v>19</v>
+      </c>
+      <c r="D23" t="str">
+        <v>CN-NMI</v>
+      </c>
+      <c r="E23" t="str">
+        <v>A320</v>
+      </c>
+      <c r="F23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>2026-05-08</v>
+      </c>
+      <c r="B24">
+        <v>2026</v>
+      </c>
+      <c r="C24">
+        <v>19</v>
+      </c>
+      <c r="D24" t="str">
+        <v>CN-NMJ</v>
+      </c>
+      <c r="E24" t="str">
+        <v>A320</v>
+      </c>
+      <c r="F24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>2026-05-08</v>
+      </c>
+      <c r="B25">
+        <v>2026</v>
+      </c>
+      <c r="C25">
+        <v>19</v>
+      </c>
+      <c r="D25" t="str">
+        <v>CN-NML</v>
+      </c>
+      <c r="E25" t="str">
+        <v>A320</v>
+      </c>
+      <c r="F25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>2026-05-08</v>
+      </c>
+      <c r="B26">
+        <v>2026</v>
+      </c>
+      <c r="C26">
+        <v>19</v>
+      </c>
+      <c r="D26" t="str">
+        <v>CN-NMN</v>
+      </c>
+      <c r="E26" t="str">
+        <v>A320</v>
+      </c>
+      <c r="F26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>2026-05-08</v>
+      </c>
+      <c r="B27">
+        <v>2026</v>
+      </c>
+      <c r="C27">
+        <v>19</v>
+      </c>
+      <c r="D27" t="str">
+        <v>CN-NMO</v>
+      </c>
+      <c r="E27" t="str">
+        <v>A320</v>
+      </c>
+      <c r="F27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>2026-05-08</v>
+      </c>
+      <c r="B28">
+        <v>2026</v>
+      </c>
+      <c r="C28">
+        <v>19</v>
+      </c>
+      <c r="D28" t="str">
+        <v>CN-NMP</v>
+      </c>
+      <c r="E28" t="str">
+        <v>A320</v>
+      </c>
+      <c r="F28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>2026-05-08</v>
+      </c>
+      <c r="B29">
+        <v>2026</v>
+      </c>
+      <c r="C29">
+        <v>19</v>
+      </c>
+      <c r="D29" t="str">
+        <v>CN-NMQ</v>
+      </c>
+      <c r="E29" t="str">
+        <v>A320</v>
+      </c>
+      <c r="F29">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>2026-05-08</v>
+      </c>
+      <c r="B30">
+        <v>2026</v>
+      </c>
+      <c r="C30">
+        <v>19</v>
+      </c>
+      <c r="D30" t="str">
+        <v>CN-NMS</v>
+      </c>
+      <c r="E30" t="str">
+        <v>A320</v>
+      </c>
+      <c r="F30">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>2026-05-08</v>
+      </c>
+      <c r="B31">
+        <v>2026</v>
+      </c>
+      <c r="C31">
+        <v>19</v>
+      </c>
+      <c r="D31" t="str">
+        <v>CN-NMT</v>
+      </c>
+      <c r="E31" t="str">
+        <v>A320</v>
+      </c>
+      <c r="F31">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F31"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>